<commit_message>
moving folders and updating investment-tradeoff
moving all workbooks to the docs folder. Updated investment trade-off analysis.md  to fall in line with the latest changes.
</commit_message>
<xml_diff>
--- a/docs/workbooks/qualified-pipe-recovery.xlsx
+++ b/docs/workbooks/qualified-pipe-recovery.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Anil\GitHub\newbridge-saas-operating-system\workbooks\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Anil\GitHub\newbridge-saas-operating-system\docs\workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ECE0DB8-BFCA-4082-9BB1-358D5449F9EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81AD932D-1F1A-4383-8955-52B64E067916}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="540" yWindow="0" windowWidth="20370" windowHeight="15480" tabRatio="715" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2595" yWindow="165" windowWidth="20370" windowHeight="15480" tabRatio="715" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRR_LP_Optimization-Initial" sheetId="2" r:id="rId1"/>
@@ -1953,7 +1953,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E7893E87-5273-4AA9-9FE1-BF0CC0642054}" type="CELLRANGE">
+                    <a:fld id="{F373BEB4-1B2A-48B0-BA54-848BFCF2B169}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1986,8 +1986,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{B28C6613-2BA1-45B8-9DD9-647BE8947837}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{07507A38-9298-48FE-A33F-DC1FF15C35A6}" type="CELLRANGE">
+                      <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
@@ -2005,6 +2005,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2019,8 +2020,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{ECAD1C57-1257-451B-B5C3-5AD8FF8789B1}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{50211899-5EE9-45EC-9AEA-EB6050E22C47}" type="CELLRANGE">
+                      <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
@@ -2038,6 +2039,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2052,8 +2054,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{10555B2E-59AA-407D-9474-9C89468B519D}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{F47CBE19-4C1C-4351-B12A-2AF50AAB1031}" type="CELLRANGE">
+                      <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
@@ -2071,6 +2073,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2085,8 +2088,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{1094A6D5-B27A-4184-8955-866DD52E7B2E}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{23FBE445-E411-4C9A-BCEB-E6C62C0C4E91}" type="CELLRANGE">
+                      <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
@@ -2104,6 +2107,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2118,8 +2122,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C54E7BCE-AFBD-4E4B-ABD3-8E127828D01B}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{74295FE2-F485-4638-9643-2ADA67DB65EE}" type="CELLRANGE">
+                      <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
@@ -2137,6 +2141,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2151,8 +2156,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{BC0D66C3-DCAE-4357-A7F5-81B4B7EAFA17}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{69A9B6E3-CD0C-49A6-B822-C694D64BF739}" type="CELLRANGE">
+                      <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
@@ -2170,6 +2175,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2266,9 +2272,9 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'LP-Scenario2-QualPipe-Scenarios'!$B$53:$B$59</c:f>
+              <c:f>'LP-Scenario2-QualPipe-Scenarios'!$G$53:$G$59</c:f>
               <c:numCache>
-                <c:formatCode>#,##0</c:formatCode>
+                <c:formatCode>#,##0.00,,"M"</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
                   <c:v>2080000</c:v>
@@ -2581,7 +2587,7 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="#,##0" sourceLinked="1"/>
+        <c:numFmt formatCode="#,##0.00,,&quot;M&quot;" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>

</xml_diff>